<commit_message>
Added AMTRAK page for INIT FAILED report, fixed some bugs, minor refactoring
</commit_message>
<xml_diff>
--- a/build/Failed_Init_Report_template.xlsx
+++ b/build/Failed_Init_Report_template.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="57398" yWindow="9338" windowWidth="19395" windowHeight="10995"/>
+    <workbookView xWindow="57398" yWindow="9338" windowWidth="19395" windowHeight="10995" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Failed Initializations.L" sheetId="1" r:id="rId1"/>
+    <sheet name="Non-Amtrak Locomotives" sheetId="1" r:id="rId1"/>
+    <sheet name="Amtrak Locomotives" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="12">
   <si>
     <t>Locomotive ID</t>
   </si>
@@ -117,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -128,6 +129,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -440,7 +444,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -467,18 +471,94 @@
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="7" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="7"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.5">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="H1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="42.3125" customWidth="1"/>
+    <col min="2" max="2" width="16.6875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.6875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.1875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.3125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.5">
+      <c r="A1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="8"/>
       <c r="J1" s="4"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.5">

</xml_diff>